<commit_message>
Add right-click batch production and tune electrolysis times
Commit the pending prototype work: right-clicking a recipe queues up to
five crafts, the queue control guards against a null item, and the two
water electrolysis recipes run in 0.4s/0.2s instead of 40s/20s.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Uranus/Dictionary/Uranus-Recipe.xlsx
+++ b/Uranus/Dictionary/Uranus-Recipe.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\CS\Uranus\Uranus\Dictionary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A98373A3-D330-41B9-8BFE-A4E1D69F79D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC7B63D3-4102-4D0D-BA97-B979B9865D2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="255" yWindow="5520" windowWidth="16350" windowHeight="15435" tabRatio="520" xr2:uid="{A23B5DB2-E4F4-4528-9DD9-79132F9B1258}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="28800" windowHeight="15435" tabRatio="520" xr2:uid="{A23B5DB2-E4F4-4528-9DD9-79132F9B1258}"/>
   </bookViews>
   <sheets>
     <sheet name="Uranus Recipe - 레시피" sheetId="2" r:id="rId1"/>
@@ -1028,7 +1028,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1036,9 +1036,6 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1">
@@ -1049,20 +1046,6 @@
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="27">
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color rgb="FF0070C0"/>
-        </left>
-        <right style="medium">
-          <color rgb="FF0070C0"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -1130,6 +1113,20 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FF0070C0"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF0070C0"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1226,40 +1223,40 @@
     <tableColumn id="9" xr3:uid="{85C863A9-7211-48F4-BF9E-257C806264E7}" uniqueName="9" name="P3C" queryTableFieldId="9"/>
     <tableColumn id="10" xr3:uid="{37712CCA-533F-4747-80D2-22D0DF4BC801}" uniqueName="10" name="P4" queryTableFieldId="10" dataDxfId="23"/>
     <tableColumn id="12" xr3:uid="{69CF101D-60E7-45E5-9C80-FED41E742B30}" uniqueName="12" name="P4C" queryTableFieldId="12"/>
-    <tableColumn id="13" xr3:uid="{F5C91EB3-F24A-458D-97B1-C0B852FC1349}" uniqueName="13" name="TIME" queryTableFieldId="13" dataDxfId="0"/>
-    <tableColumn id="14" xr3:uid="{185340F5-5679-4BDE-AD51-200EFAAA32F8}" uniqueName="14" name="M1" queryTableFieldId="14" dataDxfId="22"/>
-    <tableColumn id="15" xr3:uid="{D5050F6E-9BEB-435E-A358-7E8E0A18D56C}" uniqueName="15" name="M1C" queryTableFieldId="15" dataDxfId="21"/>
-    <tableColumn id="16" xr3:uid="{3DFB723A-FB28-4D3D-B26E-EA0950CA9C00}" uniqueName="16" name="M2" queryTableFieldId="16" dataDxfId="20"/>
-    <tableColumn id="17" xr3:uid="{85EEA9D8-45C4-4550-8F0C-D149F373DE5B}" uniqueName="17" name="M2C" queryTableFieldId="17" dataDxfId="19"/>
-    <tableColumn id="18" xr3:uid="{1E1B2F9B-5304-4B3F-95A7-98F352337FCF}" uniqueName="18" name="M3" queryTableFieldId="18" dataDxfId="18"/>
-    <tableColumn id="19" xr3:uid="{8035467C-3CAE-4ABC-8315-45D8FAE4D463}" uniqueName="19" name="M3C" queryTableFieldId="19" dataDxfId="17"/>
-    <tableColumn id="20" xr3:uid="{D73490DC-06A6-43F4-9D71-B79388DC993F}" uniqueName="20" name="M4" queryTableFieldId="20" dataDxfId="16"/>
-    <tableColumn id="21" xr3:uid="{E6FD314C-CDBA-491B-92AE-19939098ED4B}" uniqueName="21" name="M4C" queryTableFieldId="21" dataDxfId="15"/>
-    <tableColumn id="22" xr3:uid="{542730AB-5A9B-4584-9A1D-DBB90F956A1E}" uniqueName="22" name="M5" queryTableFieldId="22" dataDxfId="14"/>
-    <tableColumn id="23" xr3:uid="{FBA6C17A-E40F-4D34-B06A-46A9726626A0}" uniqueName="23" name="M5C" queryTableFieldId="23" dataDxfId="13"/>
-    <tableColumn id="24" xr3:uid="{9F13FF06-9224-4066-8999-EC882DD7B630}" uniqueName="24" name="M6" queryTableFieldId="24" dataDxfId="12"/>
+    <tableColumn id="13" xr3:uid="{F5C91EB3-F24A-458D-97B1-C0B852FC1349}" uniqueName="13" name="TIME" queryTableFieldId="13" dataDxfId="22"/>
+    <tableColumn id="14" xr3:uid="{185340F5-5679-4BDE-AD51-200EFAAA32F8}" uniqueName="14" name="M1" queryTableFieldId="14" dataDxfId="21"/>
+    <tableColumn id="15" xr3:uid="{D5050F6E-9BEB-435E-A358-7E8E0A18D56C}" uniqueName="15" name="M1C" queryTableFieldId="15" dataDxfId="20"/>
+    <tableColumn id="16" xr3:uid="{3DFB723A-FB28-4D3D-B26E-EA0950CA9C00}" uniqueName="16" name="M2" queryTableFieldId="16" dataDxfId="19"/>
+    <tableColumn id="17" xr3:uid="{85EEA9D8-45C4-4550-8F0C-D149F373DE5B}" uniqueName="17" name="M2C" queryTableFieldId="17" dataDxfId="18"/>
+    <tableColumn id="18" xr3:uid="{1E1B2F9B-5304-4B3F-95A7-98F352337FCF}" uniqueName="18" name="M3" queryTableFieldId="18" dataDxfId="17"/>
+    <tableColumn id="19" xr3:uid="{8035467C-3CAE-4ABC-8315-45D8FAE4D463}" uniqueName="19" name="M3C" queryTableFieldId="19" dataDxfId="16"/>
+    <tableColumn id="20" xr3:uid="{D73490DC-06A6-43F4-9D71-B79388DC993F}" uniqueName="20" name="M4" queryTableFieldId="20" dataDxfId="15"/>
+    <tableColumn id="21" xr3:uid="{E6FD314C-CDBA-491B-92AE-19939098ED4B}" uniqueName="21" name="M4C" queryTableFieldId="21" dataDxfId="14"/>
+    <tableColumn id="22" xr3:uid="{542730AB-5A9B-4584-9A1D-DBB90F956A1E}" uniqueName="22" name="M5" queryTableFieldId="22" dataDxfId="13"/>
+    <tableColumn id="23" xr3:uid="{FBA6C17A-E40F-4D34-B06A-46A9726626A0}" uniqueName="23" name="M5C" queryTableFieldId="23" dataDxfId="12"/>
+    <tableColumn id="24" xr3:uid="{9F13FF06-9224-4066-8999-EC882DD7B630}" uniqueName="24" name="M6" queryTableFieldId="24" dataDxfId="11"/>
     <tableColumn id="25" xr3:uid="{05E1BFCB-2B80-43BD-9CB4-09452C26078B}" uniqueName="25" name="M6C" queryTableFieldId="25"/>
-    <tableColumn id="26" xr3:uid="{CA769B84-EA50-4F5B-9590-EABC18BA0423}" uniqueName="26" name="M7" queryTableFieldId="26" dataDxfId="11"/>
+    <tableColumn id="26" xr3:uid="{CA769B84-EA50-4F5B-9590-EABC18BA0423}" uniqueName="26" name="M7" queryTableFieldId="26" dataDxfId="10"/>
     <tableColumn id="27" xr3:uid="{E727C211-3203-445C-8D58-9572D8AAB0EB}" uniqueName="27" name="M7C" queryTableFieldId="27"/>
-    <tableColumn id="28" xr3:uid="{BCB0754F-DB8F-4080-829F-178A8357B544}" uniqueName="28" name="M8" queryTableFieldId="28" dataDxfId="10"/>
+    <tableColumn id="28" xr3:uid="{BCB0754F-DB8F-4080-829F-178A8357B544}" uniqueName="28" name="M8" queryTableFieldId="28" dataDxfId="9"/>
     <tableColumn id="29" xr3:uid="{ECA145D9-2CC3-44F6-9983-B0DBB206A30F}" uniqueName="29" name="M8C" queryTableFieldId="29"/>
-    <tableColumn id="30" xr3:uid="{9A1260A8-7804-45EC-9474-8D2EEB746806}" uniqueName="30" name="M9" queryTableFieldId="30" dataDxfId="9"/>
+    <tableColumn id="30" xr3:uid="{9A1260A8-7804-45EC-9474-8D2EEB746806}" uniqueName="30" name="M9" queryTableFieldId="30" dataDxfId="8"/>
     <tableColumn id="31" xr3:uid="{7170AC84-0504-4B2E-BB86-86F015F34491}" uniqueName="31" name="M9C" queryTableFieldId="31"/>
-    <tableColumn id="32" xr3:uid="{3B421355-5E7A-4D2A-87C7-281CD11B77C6}" uniqueName="32" name="M10" queryTableFieldId="32" dataDxfId="8"/>
+    <tableColumn id="32" xr3:uid="{3B421355-5E7A-4D2A-87C7-281CD11B77C6}" uniqueName="32" name="M10" queryTableFieldId="32" dataDxfId="7"/>
     <tableColumn id="33" xr3:uid="{EB74BF48-D688-4A49-87D4-30443C383DE1}" uniqueName="33" name="M10C" queryTableFieldId="33"/>
-    <tableColumn id="34" xr3:uid="{EBBCB24C-73F6-4162-B90C-4FDA09CF229A}" uniqueName="34" name="M11" queryTableFieldId="34" dataDxfId="7"/>
+    <tableColumn id="34" xr3:uid="{EBBCB24C-73F6-4162-B90C-4FDA09CF229A}" uniqueName="34" name="M11" queryTableFieldId="34" dataDxfId="6"/>
     <tableColumn id="35" xr3:uid="{4833A826-61ED-4522-A041-A5CA2720624D}" uniqueName="35" name="M11C" queryTableFieldId="35"/>
-    <tableColumn id="36" xr3:uid="{6CCC70F0-4A97-4145-B306-7AD0FC7C2FD2}" uniqueName="36" name="M12" queryTableFieldId="36" dataDxfId="6"/>
+    <tableColumn id="36" xr3:uid="{6CCC70F0-4A97-4145-B306-7AD0FC7C2FD2}" uniqueName="36" name="M12" queryTableFieldId="36" dataDxfId="5"/>
     <tableColumn id="37" xr3:uid="{914495F1-4633-48C3-BC11-545CD6EFE6A0}" uniqueName="37" name="M12C" queryTableFieldId="37"/>
-    <tableColumn id="38" xr3:uid="{023B8C57-DF9E-476B-879A-900A3B0054E2}" uniqueName="38" name="M13" queryTableFieldId="38" dataDxfId="5"/>
+    <tableColumn id="38" xr3:uid="{023B8C57-DF9E-476B-879A-900A3B0054E2}" uniqueName="38" name="M13" queryTableFieldId="38" dataDxfId="4"/>
     <tableColumn id="39" xr3:uid="{504F7AFE-3EFA-45DD-A1CA-7A1626DB1817}" uniqueName="39" name="M13C" queryTableFieldId="39"/>
-    <tableColumn id="40" xr3:uid="{60B64089-58F4-4FEC-B015-D28FE4ED5F95}" uniqueName="40" name="M14" queryTableFieldId="40" dataDxfId="4"/>
+    <tableColumn id="40" xr3:uid="{60B64089-58F4-4FEC-B015-D28FE4ED5F95}" uniqueName="40" name="M14" queryTableFieldId="40" dataDxfId="3"/>
     <tableColumn id="41" xr3:uid="{92395F91-377A-4CFA-ADCC-E69B3B5651F4}" uniqueName="41" name="M14C" queryTableFieldId="41"/>
-    <tableColumn id="42" xr3:uid="{39E19493-1C6C-4DD5-8F11-6481E4DD2B1F}" uniqueName="42" name="M15" queryTableFieldId="42" dataDxfId="3"/>
+    <tableColumn id="42" xr3:uid="{39E19493-1C6C-4DD5-8F11-6481E4DD2B1F}" uniqueName="42" name="M15" queryTableFieldId="42" dataDxfId="2"/>
     <tableColumn id="43" xr3:uid="{20F225F4-7AC9-41B7-BF2C-AF3B1458EB08}" uniqueName="43" name="M15C" queryTableFieldId="43"/>
-    <tableColumn id="44" xr3:uid="{0C203319-91FF-4253-BFBD-683995823E93}" uniqueName="44" name="M16" queryTableFieldId="44" dataDxfId="2"/>
+    <tableColumn id="44" xr3:uid="{0C203319-91FF-4253-BFBD-683995823E93}" uniqueName="44" name="M16" queryTableFieldId="44" dataDxfId="1"/>
     <tableColumn id="45" xr3:uid="{19B23460-3FD1-4E86-9686-06EC5B3578E8}" uniqueName="45" name="M16C" queryTableFieldId="45"/>
-    <tableColumn id="46" xr3:uid="{24894DC5-C053-4813-8842-13280586F390}" uniqueName="46" name="M17" queryTableFieldId="46" dataDxfId="1"/>
+    <tableColumn id="46" xr3:uid="{24894DC5-C053-4813-8842-13280586F390}" uniqueName="46" name="M17" queryTableFieldId="46" dataDxfId="0"/>
     <tableColumn id="47" xr3:uid="{E78EA5D0-FCD9-4ED7-9A17-8FBEC24F0956}" uniqueName="47" name="M17C" queryTableFieldId="47"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1574,7 +1571,7 @@
     <col min="6" max="6" width="7.25" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="6" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7.25" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.25" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.25" style="3" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="19.75" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9.25" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="15.875" bestFit="1" customWidth="1"/>
@@ -1636,7 +1633,7 @@
       <c r="H1" t="s">
         <v>155</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>156</v>
       </c>
       <c r="J1" t="s">
@@ -1758,8 +1755,7 @@
       <c r="G2" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="3"/>
-      <c r="I2" s="4">
+      <c r="I2" s="3">
         <v>0.1</v>
       </c>
       <c r="J2" t="s">
@@ -1839,7 +1835,7 @@
       <c r="G3" t="s">
         <v>1</v>
       </c>
-      <c r="I3" s="4">
+      <c r="I3" s="3">
         <v>0.4</v>
       </c>
       <c r="J3" t="s">
@@ -1925,8 +1921,8 @@
       <c r="H4">
         <v>4</v>
       </c>
-      <c r="I4" s="4">
-        <v>40</v>
+      <c r="I4" s="3">
+        <v>0.4</v>
       </c>
       <c r="J4" t="s">
         <v>0</v>
@@ -1999,8 +1995,8 @@
       <c r="D5">
         <v>1</v>
       </c>
-      <c r="I5" s="4">
-        <v>20</v>
+      <c r="I5" s="3">
+        <v>0.2</v>
       </c>
       <c r="J5" t="s">
         <v>278</v>
@@ -2031,7 +2027,7 @@
       <c r="G6" t="s">
         <v>1</v>
       </c>
-      <c r="I6" s="4">
+      <c r="I6" s="3">
         <v>0.6</v>
       </c>
       <c r="J6" t="s">
@@ -2111,7 +2107,7 @@
       <c r="G7" t="s">
         <v>1</v>
       </c>
-      <c r="I7" s="4">
+      <c r="I7" s="3">
         <v>0.3</v>
       </c>
       <c r="J7" t="s">
@@ -2188,7 +2184,7 @@
       <c r="G8" t="s">
         <v>1</v>
       </c>
-      <c r="I8" s="4">
+      <c r="I8" s="3">
         <v>0.2</v>
       </c>
       <c r="J8" t="s">
@@ -2268,7 +2264,7 @@
       <c r="G9" t="s">
         <v>1</v>
       </c>
-      <c r="I9" s="4">
+      <c r="I9" s="3">
         <v>0.3</v>
       </c>
       <c r="J9" t="s">
@@ -2348,7 +2344,7 @@
       <c r="G10" t="s">
         <v>1</v>
       </c>
-      <c r="I10" s="4">
+      <c r="I10" s="3">
         <v>0.4</v>
       </c>
       <c r="J10" t="s">
@@ -2422,7 +2418,7 @@
       <c r="D11">
         <v>1</v>
       </c>
-      <c r="I11" s="4">
+      <c r="I11" s="3">
         <v>0.1</v>
       </c>
       <c r="J11" t="s">
@@ -2439,7 +2435,7 @@
       <c r="B12">
         <v>2</v>
       </c>
-      <c r="I12" s="4">
+      <c r="I12" s="3">
         <v>0.1</v>
       </c>
       <c r="J12" t="s">
@@ -2468,7 +2464,7 @@
       <c r="G13" t="s">
         <v>1</v>
       </c>
-      <c r="I13" s="4">
+      <c r="I13" s="3">
         <v>0.2</v>
       </c>
       <c r="J13" t="s">
@@ -2548,7 +2544,7 @@
       <c r="G14" t="s">
         <v>1</v>
       </c>
-      <c r="I14" s="4">
+      <c r="I14" s="3">
         <v>0.4</v>
       </c>
       <c r="J14" t="s">
@@ -2628,7 +2624,7 @@
       <c r="G15" t="s">
         <v>1</v>
       </c>
-      <c r="I15" s="4">
+      <c r="I15" s="3">
         <v>0.3</v>
       </c>
       <c r="J15" t="s">
@@ -2708,7 +2704,7 @@
       <c r="G16" t="s">
         <v>1</v>
       </c>
-      <c r="I16" s="4">
+      <c r="I16" s="3">
         <v>0.3</v>
       </c>
       <c r="J16" t="s">
@@ -2785,7 +2781,7 @@
       <c r="G17" t="s">
         <v>1</v>
       </c>
-      <c r="I17" s="4">
+      <c r="I17" s="3">
         <v>0.2</v>
       </c>
       <c r="J17" t="s">
@@ -2862,7 +2858,7 @@
       <c r="G18" t="s">
         <v>1</v>
       </c>
-      <c r="I18" s="4">
+      <c r="I18" s="3">
         <v>0.2</v>
       </c>
       <c r="J18" t="s">
@@ -2942,7 +2938,7 @@
       <c r="G19" t="s">
         <v>1</v>
       </c>
-      <c r="I19" s="4">
+      <c r="I19" s="3">
         <v>0.4</v>
       </c>
       <c r="J19" t="s">
@@ -3019,7 +3015,7 @@
       <c r="G20" t="s">
         <v>1</v>
       </c>
-      <c r="I20" s="4">
+      <c r="I20" s="3">
         <v>0.3</v>
       </c>
       <c r="J20" t="s">
@@ -3099,7 +3095,7 @@
       <c r="G21" t="s">
         <v>1</v>
       </c>
-      <c r="I21" s="4">
+      <c r="I21" s="3">
         <v>0.3</v>
       </c>
       <c r="J21" t="s">
@@ -3179,7 +3175,7 @@
       <c r="G22" t="s">
         <v>1</v>
       </c>
-      <c r="I22" s="4">
+      <c r="I22" s="3">
         <v>0.6</v>
       </c>
       <c r="J22" t="s">
@@ -3256,7 +3252,7 @@
       <c r="G23" t="s">
         <v>1</v>
       </c>
-      <c r="I23" s="4">
+      <c r="I23" s="3">
         <v>0.3</v>
       </c>
       <c r="J23" t="s">
@@ -3336,8 +3332,7 @@
       <c r="G24" t="s">
         <v>1</v>
       </c>
-      <c r="H24" s="3"/>
-      <c r="I24" s="4">
+      <c r="I24" s="3">
         <v>0.2</v>
       </c>
       <c r="J24" t="s">
@@ -3417,7 +3412,7 @@
       <c r="G25" t="s">
         <v>1</v>
       </c>
-      <c r="I25" s="4">
+      <c r="I25" s="3">
         <v>0.4</v>
       </c>
       <c r="J25" t="s">
@@ -3494,7 +3489,7 @@
       <c r="G26" t="s">
         <v>1</v>
       </c>
-      <c r="I26" s="4">
+      <c r="I26" s="3">
         <v>0.2</v>
       </c>
       <c r="J26" t="s">
@@ -3562,7 +3557,7 @@
       <c r="B27">
         <v>1</v>
       </c>
-      <c r="I27" s="4">
+      <c r="I27" s="3">
         <v>0.2</v>
       </c>
       <c r="J27" t="s">
@@ -3591,7 +3586,7 @@
       <c r="G28" t="s">
         <v>1</v>
       </c>
-      <c r="I28" s="4">
+      <c r="I28" s="3">
         <v>0.3</v>
       </c>
       <c r="J28" t="s">
@@ -3674,7 +3669,7 @@
       <c r="G29" t="s">
         <v>1</v>
       </c>
-      <c r="I29" s="4">
+      <c r="I29" s="3">
         <v>0.3</v>
       </c>
       <c r="J29" t="s">
@@ -3751,7 +3746,7 @@
       <c r="G30" t="s">
         <v>1</v>
       </c>
-      <c r="I30" s="4">
+      <c r="I30" s="3">
         <v>0.1</v>
       </c>
       <c r="J30" t="s">
@@ -3828,7 +3823,7 @@
       <c r="G31" t="s">
         <v>1</v>
       </c>
-      <c r="I31" s="4">
+      <c r="I31" s="3">
         <v>0.1</v>
       </c>
       <c r="J31" t="s">
@@ -3905,7 +3900,7 @@
       <c r="G32" t="s">
         <v>1</v>
       </c>
-      <c r="I32" s="4">
+      <c r="I32" s="3">
         <v>0.2</v>
       </c>
       <c r="J32" t="s">
@@ -3982,7 +3977,7 @@
       <c r="G33" t="s">
         <v>1</v>
       </c>
-      <c r="I33" s="4">
+      <c r="I33" s="3">
         <v>0.1</v>
       </c>
       <c r="J33" t="s">
@@ -4059,7 +4054,7 @@
       <c r="G34" t="s">
         <v>1</v>
       </c>
-      <c r="I34" s="4">
+      <c r="I34" s="3">
         <v>0.1</v>
       </c>
       <c r="J34" t="s">
@@ -4142,7 +4137,7 @@
       <c r="G35" t="s">
         <v>1</v>
       </c>
-      <c r="I35" s="4">
+      <c r="I35" s="3">
         <v>0.03</v>
       </c>
       <c r="J35" t="s">
@@ -7047,7 +7042,7 @@
       <c r="G73" t="s">
         <v>1</v>
       </c>
-      <c r="I73" s="4">
+      <c r="I73" s="3">
         <v>5</v>
       </c>
       <c r="J73" t="s">
@@ -7118,7 +7113,7 @@
       <c r="B74">
         <v>1</v>
       </c>
-      <c r="I74" s="4">
+      <c r="I74" s="3">
         <v>4</v>
       </c>
       <c r="J74" t="s">
@@ -7153,7 +7148,7 @@
       <c r="B75">
         <v>1</v>
       </c>
-      <c r="I75" s="4">
+      <c r="I75" s="3">
         <v>5</v>
       </c>
       <c r="J75" t="s">
@@ -7194,7 +7189,7 @@
       <c r="B76">
         <v>1</v>
       </c>
-      <c r="I76" s="4">
+      <c r="I76" s="3">
         <v>6</v>
       </c>
       <c r="J76" t="s">
@@ -7235,7 +7230,7 @@
       <c r="B77">
         <v>1</v>
       </c>
-      <c r="I77" s="4">
+      <c r="I77" s="3">
         <v>7</v>
       </c>
       <c r="J77" t="s">
@@ -7276,7 +7271,7 @@
       <c r="B78">
         <v>1</v>
       </c>
-      <c r="I78" s="4">
+      <c r="I78" s="3">
         <v>5</v>
       </c>
       <c r="J78" t="s">
@@ -7311,7 +7306,7 @@
       <c r="B79">
         <v>1</v>
       </c>
-      <c r="I79" s="4">
+      <c r="I79" s="3">
         <v>6</v>
       </c>
       <c r="J79" t="s">
@@ -7346,7 +7341,7 @@
       <c r="B80">
         <v>1</v>
       </c>
-      <c r="I80" s="4">
+      <c r="I80" s="3">
         <v>5</v>
       </c>
       <c r="J80" t="s">
@@ -7381,7 +7376,7 @@
       <c r="B81">
         <v>1</v>
       </c>
-      <c r="I81" s="4">
+      <c r="I81" s="3">
         <v>4</v>
       </c>
       <c r="J81" t="s">
@@ -7410,7 +7405,7 @@
       <c r="B82">
         <v>1</v>
       </c>
-      <c r="I82" s="4">
+      <c r="I82" s="3">
         <v>6</v>
       </c>
       <c r="J82" t="s">
@@ -7445,7 +7440,7 @@
       <c r="B83">
         <v>1</v>
       </c>
-      <c r="I83" s="4">
+      <c r="I83" s="3">
         <v>7</v>
       </c>
       <c r="J83" t="s">
@@ -7480,7 +7475,7 @@
       <c r="B84">
         <v>1</v>
       </c>
-      <c r="I84" s="4">
+      <c r="I84" s="3">
         <v>5</v>
       </c>
       <c r="J84" t="s">
@@ -7509,7 +7504,7 @@
       <c r="B85">
         <v>1</v>
       </c>
-      <c r="I85" s="4">
+      <c r="I85" s="3">
         <v>8</v>
       </c>
       <c r="J85" t="s">
@@ -7556,7 +7551,7 @@
       <c r="B86">
         <v>1</v>
       </c>
-      <c r="I86" s="4">
+      <c r="I86" s="3">
         <v>6</v>
       </c>
       <c r="J86" t="s">
@@ -7591,7 +7586,7 @@
       <c r="B87">
         <v>1</v>
       </c>
-      <c r="I87" s="4">
+      <c r="I87" s="3">
         <v>4</v>
       </c>
       <c r="J87" t="s">
@@ -7620,7 +7615,7 @@
       <c r="B88">
         <v>1</v>
       </c>
-      <c r="I88" s="4">
+      <c r="I88" s="3">
         <v>5</v>
       </c>
       <c r="J88" t="s">
@@ -7655,7 +7650,7 @@
       <c r="B89">
         <v>1</v>
       </c>
-      <c r="I89" s="4">
+      <c r="I89" s="3">
         <v>6</v>
       </c>
       <c r="J89" t="s">
@@ -7690,7 +7685,7 @@
       <c r="B90">
         <v>1</v>
       </c>
-      <c r="I90" s="4">
+      <c r="I90" s="3">
         <v>20</v>
       </c>
       <c r="J90" t="s">
@@ -7725,7 +7720,7 @@
       <c r="B91">
         <v>1</v>
       </c>
-      <c r="I91" s="4">
+      <c r="I91" s="3">
         <v>5</v>
       </c>
       <c r="J91" t="s">
@@ -7754,7 +7749,7 @@
       <c r="B92">
         <v>1</v>
       </c>
-      <c r="I92" s="4">
+      <c r="I92" s="3">
         <v>4</v>
       </c>
       <c r="J92" t="s">
@@ -7783,7 +7778,7 @@
       <c r="B93">
         <v>1</v>
       </c>
-      <c r="I93" s="4">
+      <c r="I93" s="3">
         <v>86</v>
       </c>
       <c r="J93" t="s">
@@ -7800,7 +7795,7 @@
       <c r="B94">
         <v>1</v>
       </c>
-      <c r="I94" s="4">
+      <c r="I94" s="3">
         <v>6</v>
       </c>
       <c r="J94" t="s">
@@ -7830,7 +7825,7 @@
       <c r="B95">
         <v>1</v>
       </c>
-      <c r="I95" s="4">
+      <c r="I95" s="3">
         <v>10</v>
       </c>
       <c r="J95" t="s">
@@ -7866,7 +7861,7 @@
       <c r="B96">
         <v>1</v>
       </c>
-      <c r="I96" s="4">
+      <c r="I96" s="3">
         <v>12</v>
       </c>
       <c r="J96" t="s">
@@ -7908,7 +7903,7 @@
       <c r="B97">
         <v>1</v>
       </c>
-      <c r="I97" s="4">
+      <c r="I97" s="3">
         <v>15</v>
       </c>
       <c r="J97" t="s">
@@ -7950,7 +7945,7 @@
       <c r="B98">
         <v>1</v>
       </c>
-      <c r="I98" s="4">
+      <c r="I98" s="3">
         <v>10</v>
       </c>
       <c r="J98" t="s">
@@ -7992,7 +7987,7 @@
       <c r="B99">
         <v>1</v>
       </c>
-      <c r="I99" s="4">
+      <c r="I99" s="3">
         <v>8</v>
       </c>
       <c r="J99" t="s">
@@ -8034,7 +8029,7 @@
       <c r="B100">
         <v>1</v>
       </c>
-      <c r="I100" s="4">
+      <c r="I100" s="3">
         <v>5</v>
       </c>
       <c r="J100" t="s">
@@ -8058,7 +8053,7 @@
       <c r="B101">
         <v>1</v>
       </c>
-      <c r="I101" s="4">
+      <c r="I101" s="3">
         <v>8</v>
       </c>
       <c r="J101" t="s">
@@ -8088,7 +8083,7 @@
       <c r="B102">
         <v>600</v>
       </c>
-      <c r="I102" s="4">
+      <c r="I102" s="3">
         <v>10</v>
       </c>
       <c r="J102" t="s">
@@ -8117,7 +8112,7 @@
       <c r="B103">
         <v>250</v>
       </c>
-      <c r="I103" s="4">
+      <c r="I103" s="3">
         <v>60</v>
       </c>
       <c r="J103" t="s">
@@ -8146,7 +8141,7 @@
       <c r="B104">
         <v>36</v>
       </c>
-      <c r="I104" s="4">
+      <c r="I104" s="3">
         <v>2</v>
       </c>
       <c r="J104" t="s">
@@ -8169,7 +8164,7 @@
       <c r="B105">
         <v>300</v>
       </c>
-      <c r="I105" s="4">
+      <c r="I105" s="3">
         <v>10</v>
       </c>
       <c r="J105" t="s">
@@ -8198,7 +8193,7 @@
       <c r="B106">
         <v>1200</v>
       </c>
-      <c r="I106" s="4">
+      <c r="I106" s="3">
         <v>100</v>
       </c>
       <c r="J106" t="s">
@@ -8227,7 +8222,7 @@
       <c r="B107">
         <v>1600</v>
       </c>
-      <c r="I107" s="4">
+      <c r="I107" s="3">
         <v>20</v>
       </c>
       <c r="J107" t="s">
@@ -8250,7 +8245,7 @@
       <c r="B108">
         <v>4500</v>
       </c>
-      <c r="I108" s="4">
+      <c r="I108" s="3">
         <v>30</v>
       </c>
       <c r="J108" t="s">
@@ -8273,7 +8268,7 @@
       <c r="B109">
         <v>10000</v>
       </c>
-      <c r="I109" s="4">
+      <c r="I109" s="3">
         <v>200</v>
       </c>
       <c r="J109" t="s">
@@ -8296,7 +8291,7 @@
       <c r="B110">
         <v>150</v>
       </c>
-      <c r="I110" s="4">
+      <c r="I110" s="3">
         <v>5</v>
       </c>
       <c r="J110" t="s">
@@ -8319,7 +8314,7 @@
       <c r="B111">
         <v>180</v>
       </c>
-      <c r="I111" s="4">
+      <c r="I111" s="3">
         <v>6</v>
       </c>
       <c r="J111" t="s">

</xml_diff>